<commit_message>
added function signature to doc
</commit_message>
<xml_diff>
--- a/Docs/Lab02/Lab02_BBT_TCs_Form.xlsx
+++ b/Docs/Lab02/Lab02_BBT_TCs_Form.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="28526"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A0CEC025-83EE-44C9-BB65-F1879B49C42A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{724B0AA4-A034-430C-B939-B65F45FF22CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" firstSheet="3" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -13,7 +13,7 @@
     <sheet name="F01.BVA" sheetId="3" r:id="rId3"/>
     <sheet name="BBT-TCs" sheetId="4" r:id="rId4"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -117,7 +117,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="313" uniqueCount="156">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="319" uniqueCount="162">
   <si>
     <t>VVSS, Info Romana, 2024-2025</t>
   </si>
@@ -751,6 +751,24 @@
   </si>
   <si>
     <t>DOUBLE_MAX</t>
+  </si>
+  <si>
+    <t>Functie testata:</t>
+  </si>
+  <si>
+    <t>public void addOutsourcePart(String name, double price, int inStock, int min, int  max, String partDynamicValue)</t>
+  </si>
+  <si>
+    <t>preconditii:</t>
+  </si>
+  <si>
+    <t>name, partDynamicValue - sir de caractere</t>
+  </si>
+  <si>
+    <t>inStock, min, max ∈ ℕ; min &lt;= inStock &lt;= max</t>
+  </si>
+  <si>
+    <t>price ∈ ℝ+</t>
   </si>
 </sst>
 </file>
@@ -1571,86 +1589,113 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1658,35 +1703,20 @@
     <xf numFmtId="0" fontId="19" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="29" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1694,30 +1724,78 @@
     <xf numFmtId="0" fontId="29" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="2" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1725,66 +1803,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="3" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="3" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="2" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -2335,35 +2353,35 @@
       <c r="E1" s="54"/>
     </row>
     <row r="3" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B3" s="74" t="s">
+      <c r="B3" s="59" t="s">
         <v>14</v>
       </c>
-      <c r="C3" s="75"/>
-      <c r="D3" s="75"/>
-      <c r="E3" s="75"/>
-      <c r="F3" s="75"/>
-      <c r="G3" s="76"/>
+      <c r="C3" s="60"/>
+      <c r="D3" s="60"/>
+      <c r="E3" s="60"/>
+      <c r="F3" s="60"/>
+      <c r="G3" s="61"/>
     </row>
     <row r="5" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B5" s="77" t="s">
+      <c r="B5" s="62" t="s">
         <v>22</v>
       </c>
-      <c r="C5" s="77"/>
-      <c r="D5" s="77"/>
-      <c r="E5" s="77"/>
-      <c r="G5" s="78" t="s">
+      <c r="C5" s="62"/>
+      <c r="D5" s="62"/>
+      <c r="E5" s="62"/>
+      <c r="G5" s="63" t="s">
         <v>23</v>
       </c>
-      <c r="H5" s="78"/>
-      <c r="I5" s="78"/>
-      <c r="J5" s="78"/>
-      <c r="K5" s="78"/>
-      <c r="L5" s="78"/>
-      <c r="M5" s="78"/>
-      <c r="N5" s="78"/>
-      <c r="O5" s="78"/>
-      <c r="P5" s="78"/>
-      <c r="Q5" s="78"/>
+      <c r="H5" s="63"/>
+      <c r="I5" s="63"/>
+      <c r="J5" s="63"/>
+      <c r="K5" s="63"/>
+      <c r="L5" s="63"/>
+      <c r="M5" s="63"/>
+      <c r="N5" s="63"/>
+      <c r="O5" s="63"/>
+      <c r="P5" s="63"/>
+      <c r="Q5" s="63"/>
     </row>
     <row r="6" spans="2:17" x14ac:dyDescent="0.25">
       <c r="B6" s="19" t="s">
@@ -2378,39 +2396,39 @@
       <c r="E6" s="19" t="s">
         <v>27</v>
       </c>
-      <c r="G6" s="79" t="s">
+      <c r="G6" s="64" t="s">
         <v>28</v>
       </c>
-      <c r="H6" s="63" t="s">
+      <c r="H6" s="78" t="s">
         <v>29</v>
       </c>
-      <c r="I6" s="61" t="s">
+      <c r="I6" s="76" t="s">
         <v>30</v>
       </c>
-      <c r="J6" s="66"/>
-      <c r="K6" s="66"/>
-      <c r="L6" s="66"/>
-      <c r="M6" s="66"/>
-      <c r="N6" s="66"/>
-      <c r="O6" s="62"/>
-      <c r="P6" s="65" t="s">
+      <c r="J6" s="81"/>
+      <c r="K6" s="81"/>
+      <c r="L6" s="81"/>
+      <c r="M6" s="81"/>
+      <c r="N6" s="81"/>
+      <c r="O6" s="77"/>
+      <c r="P6" s="80" t="s">
         <v>31</v>
       </c>
-      <c r="Q6" s="65"/>
+      <c r="Q6" s="80"/>
     </row>
     <row r="7" spans="2:17" x14ac:dyDescent="0.25">
       <c r="B7" s="4">
         <v>1</v>
       </c>
-      <c r="C7" s="71" t="s">
+      <c r="C7" s="56" t="s">
         <v>32</v>
       </c>
       <c r="D7" s="4" t="s">
         <v>32</v>
       </c>
       <c r="E7" s="4"/>
-      <c r="G7" s="80"/>
-      <c r="H7" s="64"/>
+      <c r="G7" s="65"/>
+      <c r="H7" s="79"/>
       <c r="I7" s="19" t="s">
         <v>33</v>
       </c>
@@ -2426,20 +2444,20 @@
       <c r="M7" s="19" t="s">
         <v>37</v>
       </c>
-      <c r="N7" s="61" t="s">
+      <c r="N7" s="76" t="s">
         <v>38</v>
       </c>
-      <c r="O7" s="62"/>
-      <c r="P7" s="61" t="s">
+      <c r="O7" s="77"/>
+      <c r="P7" s="76" t="s">
         <v>39</v>
       </c>
-      <c r="Q7" s="62"/>
+      <c r="Q7" s="77"/>
     </row>
     <row r="8" spans="2:17" x14ac:dyDescent="0.25">
       <c r="B8" s="4">
         <v>2</v>
       </c>
-      <c r="C8" s="71"/>
+      <c r="C8" s="56"/>
       <c r="D8" s="4"/>
       <c r="E8" s="4" t="s">
         <v>40</v>
@@ -2465,22 +2483,22 @@
       <c r="M8" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="N8" s="57" t="s">
+      <c r="N8" s="74" t="s">
         <v>46</v>
       </c>
-      <c r="O8" s="58" t="s">
+      <c r="O8" s="75" t="s">
         <v>47</v>
       </c>
-      <c r="P8" s="57" t="s">
+      <c r="P8" s="74" t="s">
         <v>48</v>
       </c>
-      <c r="Q8" s="58"/>
+      <c r="Q8" s="75"/>
     </row>
     <row r="9" spans="2:17" x14ac:dyDescent="0.25">
       <c r="B9" s="4">
         <v>3</v>
       </c>
-      <c r="C9" s="71" t="s">
+      <c r="C9" s="56" t="s">
         <v>49</v>
       </c>
       <c r="D9" s="4" t="s">
@@ -2508,22 +2526,22 @@
       <c r="M9" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="N9" s="57" t="s">
+      <c r="N9" s="74" t="s">
         <v>50</v>
       </c>
-      <c r="O9" s="58" t="s">
+      <c r="O9" s="75" t="s">
         <v>52</v>
       </c>
-      <c r="P9" s="57" t="s">
+      <c r="P9" s="74" t="s">
         <v>50</v>
       </c>
-      <c r="Q9" s="58"/>
+      <c r="Q9" s="75"/>
     </row>
     <row r="10" spans="2:17" x14ac:dyDescent="0.25">
       <c r="B10" s="4">
         <v>4</v>
       </c>
-      <c r="C10" s="71"/>
+      <c r="C10" s="56"/>
       <c r="D10" s="4"/>
       <c r="E10" s="4" t="s">
         <v>53</v>
@@ -2549,20 +2567,20 @@
       <c r="M10" s="11" t="s">
         <v>45</v>
       </c>
-      <c r="N10" s="69" t="s">
+      <c r="N10" s="68" t="s">
         <v>46</v>
       </c>
-      <c r="O10" s="70"/>
-      <c r="P10" s="69" t="s">
+      <c r="O10" s="69"/>
+      <c r="P10" s="68" t="s">
         <v>56</v>
       </c>
-      <c r="Q10" s="70"/>
+      <c r="Q10" s="69"/>
     </row>
     <row r="11" spans="2:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B11" s="4">
         <v>5</v>
       </c>
-      <c r="C11" s="71" t="s">
+      <c r="C11" s="56" t="s">
         <v>57</v>
       </c>
       <c r="D11" s="4" t="s">
@@ -2590,20 +2608,20 @@
       <c r="M11" s="11" t="s">
         <v>50</v>
       </c>
-      <c r="N11" s="69" t="s">
+      <c r="N11" s="68" t="s">
         <v>50</v>
       </c>
-      <c r="O11" s="70"/>
-      <c r="P11" s="69" t="s">
+      <c r="O11" s="69"/>
+      <c r="P11" s="68" t="s">
         <v>50</v>
       </c>
-      <c r="Q11" s="70"/>
+      <c r="Q11" s="69"/>
     </row>
     <row r="12" spans="2:17" x14ac:dyDescent="0.25">
       <c r="B12" s="4">
         <v>6</v>
       </c>
-      <c r="C12" s="71"/>
+      <c r="C12" s="56"/>
       <c r="D12" s="4"/>
       <c r="E12" s="4" t="s">
         <v>59</v>
@@ -2633,16 +2651,16 @@
         <v>46</v>
       </c>
       <c r="O12" s="6"/>
-      <c r="P12" s="67" t="s">
+      <c r="P12" s="70" t="s">
         <v>62</v>
       </c>
-      <c r="Q12" s="68"/>
+      <c r="Q12" s="71"/>
     </row>
     <row r="13" spans="2:17" x14ac:dyDescent="0.25">
       <c r="B13" s="4">
         <v>7</v>
       </c>
-      <c r="C13" s="72" t="s">
+      <c r="C13" s="57" t="s">
         <v>63</v>
       </c>
       <c r="D13" s="4" t="s">
@@ -2670,20 +2688,20 @@
       <c r="M13" s="6" t="s">
         <v>50</v>
       </c>
-      <c r="N13" s="67" t="s">
+      <c r="N13" s="70" t="s">
         <v>50</v>
       </c>
-      <c r="O13" s="68"/>
-      <c r="P13" s="67" t="s">
+      <c r="O13" s="71"/>
+      <c r="P13" s="70" t="s">
         <v>50</v>
       </c>
-      <c r="Q13" s="68"/>
+      <c r="Q13" s="71"/>
     </row>
     <row r="14" spans="2:17" x14ac:dyDescent="0.25">
       <c r="B14" s="4">
         <v>8</v>
       </c>
-      <c r="C14" s="73"/>
+      <c r="C14" s="58"/>
       <c r="D14" s="4"/>
       <c r="E14" s="4" t="s">
         <v>64</v>
@@ -2709,18 +2727,18 @@
       <c r="M14" s="14" t="s">
         <v>65</v>
       </c>
-      <c r="N14" s="81" t="s">
+      <c r="N14" s="66" t="s">
         <v>65</v>
       </c>
-      <c r="O14" s="82"/>
-      <c r="P14" s="59"/>
-      <c r="Q14" s="60"/>
+      <c r="O14" s="67"/>
+      <c r="P14" s="72"/>
+      <c r="Q14" s="73"/>
     </row>
     <row r="15" spans="2:17" x14ac:dyDescent="0.25">
       <c r="B15" s="4">
         <v>9</v>
       </c>
-      <c r="C15" s="71" t="s">
+      <c r="C15" s="56" t="s">
         <v>50</v>
       </c>
       <c r="D15" s="4"/>
@@ -2736,16 +2754,16 @@
       <c r="K15" s="14"/>
       <c r="L15" s="14"/>
       <c r="M15" s="14"/>
-      <c r="N15" s="57"/>
-      <c r="O15" s="58"/>
-      <c r="P15" s="59"/>
-      <c r="Q15" s="60"/>
+      <c r="N15" s="74"/>
+      <c r="O15" s="75"/>
+      <c r="P15" s="72"/>
+      <c r="Q15" s="73"/>
     </row>
     <row r="16" spans="2:17" x14ac:dyDescent="0.25">
       <c r="B16" s="4">
         <v>10</v>
       </c>
-      <c r="C16" s="71"/>
+      <c r="C16" s="56"/>
       <c r="D16" s="4"/>
       <c r="E16" s="4"/>
       <c r="G16" s="15"/>
@@ -2755,16 +2773,16 @@
       <c r="K16" s="14"/>
       <c r="L16" s="14"/>
       <c r="M16" s="14"/>
-      <c r="N16" s="57"/>
-      <c r="O16" s="58"/>
-      <c r="P16" s="59"/>
-      <c r="Q16" s="60"/>
+      <c r="N16" s="74"/>
+      <c r="O16" s="75"/>
+      <c r="P16" s="72"/>
+      <c r="Q16" s="73"/>
     </row>
     <row r="17" spans="2:17" x14ac:dyDescent="0.25">
       <c r="B17" s="4">
         <v>11</v>
       </c>
-      <c r="C17" s="71" t="s">
+      <c r="C17" s="56" t="s">
         <v>50</v>
       </c>
       <c r="D17" s="4"/>
@@ -2776,16 +2794,16 @@
       <c r="K17" s="14"/>
       <c r="L17" s="14"/>
       <c r="M17" s="14"/>
-      <c r="N17" s="57"/>
-      <c r="O17" s="58"/>
-      <c r="P17" s="59"/>
-      <c r="Q17" s="60"/>
+      <c r="N17" s="74"/>
+      <c r="O17" s="75"/>
+      <c r="P17" s="72"/>
+      <c r="Q17" s="73"/>
     </row>
     <row r="18" spans="2:17" x14ac:dyDescent="0.25">
       <c r="B18" s="4">
         <v>12</v>
       </c>
-      <c r="C18" s="71"/>
+      <c r="C18" s="56"/>
       <c r="D18" s="4"/>
       <c r="E18" s="4"/>
       <c r="G18" s="15"/>
@@ -2795,16 +2813,16 @@
       <c r="K18" s="14"/>
       <c r="L18" s="14"/>
       <c r="M18" s="14"/>
-      <c r="N18" s="57"/>
-      <c r="O18" s="58"/>
-      <c r="P18" s="59"/>
-      <c r="Q18" s="60"/>
+      <c r="N18" s="74"/>
+      <c r="O18" s="75"/>
+      <c r="P18" s="72"/>
+      <c r="Q18" s="73"/>
     </row>
     <row r="19" spans="2:17" x14ac:dyDescent="0.25">
       <c r="B19" s="4">
         <v>13</v>
       </c>
-      <c r="C19" s="71" t="s">
+      <c r="C19" s="56" t="s">
         <v>50</v>
       </c>
       <c r="D19" s="4"/>
@@ -2816,16 +2834,16 @@
       <c r="K19" s="2"/>
       <c r="L19" s="2"/>
       <c r="M19" s="2"/>
-      <c r="N19" s="57"/>
-      <c r="O19" s="58"/>
-      <c r="P19" s="59"/>
-      <c r="Q19" s="60"/>
+      <c r="N19" s="74"/>
+      <c r="O19" s="75"/>
+      <c r="P19" s="72"/>
+      <c r="Q19" s="73"/>
     </row>
     <row r="20" spans="2:17" x14ac:dyDescent="0.25">
       <c r="B20" s="4">
         <v>14</v>
       </c>
-      <c r="C20" s="71"/>
+      <c r="C20" s="56"/>
       <c r="D20" s="4"/>
       <c r="E20" s="4"/>
     </row>
@@ -2833,11 +2851,36 @@
       <c r="D22" t="s">
         <v>66</v>
       </c>
-      <c r="F22" s="56"/>
-      <c r="G22" s="56"/>
+      <c r="F22" s="82"/>
+      <c r="G22" s="82"/>
     </row>
   </sheetData>
   <mergeCells count="41">
+    <mergeCell ref="F22:G22"/>
+    <mergeCell ref="N15:O15"/>
+    <mergeCell ref="N16:O16"/>
+    <mergeCell ref="N17:O17"/>
+    <mergeCell ref="P16:Q16"/>
+    <mergeCell ref="P17:Q17"/>
+    <mergeCell ref="N19:O19"/>
+    <mergeCell ref="P18:Q18"/>
+    <mergeCell ref="P19:Q19"/>
+    <mergeCell ref="N18:O18"/>
+    <mergeCell ref="P15:Q15"/>
+    <mergeCell ref="P8:Q8"/>
+    <mergeCell ref="P9:Q9"/>
+    <mergeCell ref="N7:O7"/>
+    <mergeCell ref="H6:H7"/>
+    <mergeCell ref="P6:Q6"/>
+    <mergeCell ref="N9:O9"/>
+    <mergeCell ref="I6:O6"/>
+    <mergeCell ref="N8:O8"/>
+    <mergeCell ref="P7:Q7"/>
+    <mergeCell ref="P13:Q13"/>
+    <mergeCell ref="P14:Q14"/>
+    <mergeCell ref="N13:O13"/>
+    <mergeCell ref="N10:O10"/>
+    <mergeCell ref="N11:O11"/>
     <mergeCell ref="B1:E1"/>
     <mergeCell ref="C19:C20"/>
     <mergeCell ref="C7:C8"/>
@@ -2854,31 +2897,6 @@
     <mergeCell ref="P10:Q10"/>
     <mergeCell ref="P11:Q11"/>
     <mergeCell ref="P12:Q12"/>
-    <mergeCell ref="P13:Q13"/>
-    <mergeCell ref="P14:Q14"/>
-    <mergeCell ref="N13:O13"/>
-    <mergeCell ref="N10:O10"/>
-    <mergeCell ref="N11:O11"/>
-    <mergeCell ref="P8:Q8"/>
-    <mergeCell ref="P9:Q9"/>
-    <mergeCell ref="N7:O7"/>
-    <mergeCell ref="H6:H7"/>
-    <mergeCell ref="P6:Q6"/>
-    <mergeCell ref="N9:O9"/>
-    <mergeCell ref="I6:O6"/>
-    <mergeCell ref="N8:O8"/>
-    <mergeCell ref="P7:Q7"/>
-    <mergeCell ref="F22:G22"/>
-    <mergeCell ref="N15:O15"/>
-    <mergeCell ref="N16:O16"/>
-    <mergeCell ref="N17:O17"/>
-    <mergeCell ref="P16:Q16"/>
-    <mergeCell ref="P17:Q17"/>
-    <mergeCell ref="N19:O19"/>
-    <mergeCell ref="P18:Q18"/>
-    <mergeCell ref="P19:Q19"/>
-    <mergeCell ref="N18:O18"/>
-    <mergeCell ref="P15:Q15"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -2919,14 +2937,14 @@
       <c r="E1" s="54"/>
     </row>
     <row r="3" spans="2:18" x14ac:dyDescent="0.25">
-      <c r="B3" s="74" t="s">
+      <c r="B3" s="59" t="s">
         <v>14</v>
       </c>
-      <c r="C3" s="75"/>
-      <c r="D3" s="75"/>
-      <c r="E3" s="75"/>
-      <c r="F3" s="75"/>
-      <c r="G3" s="76"/>
+      <c r="C3" s="60"/>
+      <c r="D3" s="60"/>
+      <c r="E3" s="60"/>
+      <c r="F3" s="60"/>
+      <c r="G3" s="61"/>
     </row>
     <row r="5" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B5" s="89" t="s">
@@ -2935,20 +2953,20 @@
       <c r="C5" s="89"/>
       <c r="D5" s="89"/>
       <c r="E5" s="3"/>
-      <c r="G5" s="78" t="s">
+      <c r="G5" s="63" t="s">
         <v>68</v>
       </c>
-      <c r="H5" s="78"/>
-      <c r="I5" s="78"/>
-      <c r="J5" s="78"/>
-      <c r="K5" s="78"/>
-      <c r="L5" s="78"/>
-      <c r="M5" s="78"/>
-      <c r="N5" s="78"/>
-      <c r="O5" s="78"/>
-      <c r="P5" s="78"/>
-      <c r="Q5" s="78"/>
-      <c r="R5" s="78"/>
+      <c r="H5" s="63"/>
+      <c r="I5" s="63"/>
+      <c r="J5" s="63"/>
+      <c r="K5" s="63"/>
+      <c r="L5" s="63"/>
+      <c r="M5" s="63"/>
+      <c r="N5" s="63"/>
+      <c r="O5" s="63"/>
+      <c r="P5" s="63"/>
+      <c r="Q5" s="63"/>
+      <c r="R5" s="63"/>
     </row>
     <row r="6" spans="2:18" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B6" s="4" t="s">
@@ -2961,45 +2979,45 @@
         <v>67</v>
       </c>
       <c r="E6" s="7"/>
-      <c r="G6" s="79" t="s">
+      <c r="G6" s="64" t="s">
         <v>70</v>
       </c>
-      <c r="H6" s="79" t="s">
+      <c r="H6" s="64" t="s">
         <v>71</v>
       </c>
-      <c r="I6" s="79" t="s">
+      <c r="I6" s="64" t="s">
         <v>72</v>
       </c>
-      <c r="J6" s="63" t="s">
+      <c r="J6" s="78" t="s">
         <v>73</v>
       </c>
-      <c r="K6" s="85" t="s">
+      <c r="K6" s="90" t="s">
         <v>30</v>
       </c>
-      <c r="L6" s="86"/>
-      <c r="M6" s="86"/>
-      <c r="N6" s="86"/>
-      <c r="O6" s="86"/>
-      <c r="P6" s="87"/>
-      <c r="Q6" s="85" t="s">
+      <c r="L6" s="94"/>
+      <c r="M6" s="94"/>
+      <c r="N6" s="94"/>
+      <c r="O6" s="94"/>
+      <c r="P6" s="91"/>
+      <c r="Q6" s="90" t="s">
         <v>31</v>
       </c>
-      <c r="R6" s="87"/>
+      <c r="R6" s="91"/>
     </row>
     <row r="7" spans="2:18" ht="45" x14ac:dyDescent="0.25">
-      <c r="B7" s="72">
+      <c r="B7" s="57">
         <v>1</v>
       </c>
-      <c r="C7" s="91" t="s">
+      <c r="C7" s="84" t="s">
         <v>74</v>
       </c>
       <c r="D7" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="G7" s="80"/>
-      <c r="H7" s="80"/>
-      <c r="I7" s="80"/>
-      <c r="J7" s="64"/>
+      <c r="G7" s="65"/>
+      <c r="H7" s="65"/>
+      <c r="I7" s="65"/>
+      <c r="J7" s="79"/>
       <c r="K7" s="19" t="s">
         <v>33</v>
       </c>
@@ -3018,14 +3036,14 @@
       <c r="P7" s="19" t="s">
         <v>38</v>
       </c>
-      <c r="Q7" s="61" t="s">
+      <c r="Q7" s="76" t="s">
         <v>76</v>
       </c>
-      <c r="R7" s="62"/>
+      <c r="R7" s="77"/>
     </row>
     <row r="8" spans="2:18" x14ac:dyDescent="0.25">
-      <c r="B8" s="90"/>
-      <c r="C8" s="92"/>
+      <c r="B8" s="83"/>
+      <c r="C8" s="85"/>
       <c r="D8" s="2" t="s">
         <v>77</v>
       </c>
@@ -3045,12 +3063,12 @@
       <c r="N8" s="30"/>
       <c r="O8" s="30"/>
       <c r="P8" s="30"/>
-      <c r="Q8" s="83"/>
-      <c r="R8" s="84"/>
+      <c r="Q8" s="92"/>
+      <c r="R8" s="93"/>
     </row>
     <row r="9" spans="2:18" x14ac:dyDescent="0.25">
-      <c r="B9" s="90"/>
-      <c r="C9" s="92"/>
+      <c r="B9" s="83"/>
+      <c r="C9" s="85"/>
       <c r="D9" s="2" t="s">
         <v>79</v>
       </c>
@@ -3080,14 +3098,14 @@
       <c r="P9" s="14" t="s">
         <v>50</v>
       </c>
-      <c r="Q9" s="67" t="s">
+      <c r="Q9" s="70" t="s">
         <v>62</v>
       </c>
-      <c r="R9" s="68"/>
+      <c r="R9" s="71"/>
     </row>
     <row r="10" spans="2:18" x14ac:dyDescent="0.25">
-      <c r="B10" s="90"/>
-      <c r="C10" s="92"/>
+      <c r="B10" s="83"/>
+      <c r="C10" s="85"/>
       <c r="D10" s="2" t="s">
         <v>81</v>
       </c>
@@ -3117,14 +3135,14 @@
       <c r="P10" s="30" t="s">
         <v>46</v>
       </c>
-      <c r="Q10" s="83" t="s">
+      <c r="Q10" s="92" t="s">
         <v>48</v>
       </c>
-      <c r="R10" s="84"/>
+      <c r="R10" s="93"/>
     </row>
     <row r="11" spans="2:18" x14ac:dyDescent="0.25">
-      <c r="B11" s="90"/>
-      <c r="C11" s="92"/>
+      <c r="B11" s="83"/>
+      <c r="C11" s="85"/>
       <c r="D11" s="2" t="s">
         <v>85</v>
       </c>
@@ -3154,14 +3172,14 @@
       <c r="P11" s="30" t="s">
         <v>46</v>
       </c>
-      <c r="Q11" s="83" t="s">
+      <c r="Q11" s="92" t="s">
         <v>48</v>
       </c>
-      <c r="R11" s="84"/>
+      <c r="R11" s="93"/>
     </row>
     <row r="12" spans="2:18" x14ac:dyDescent="0.25">
-      <c r="B12" s="73"/>
-      <c r="C12" s="93"/>
+      <c r="B12" s="58"/>
+      <c r="C12" s="86"/>
       <c r="D12" s="2" t="s">
         <v>87</v>
       </c>
@@ -3191,16 +3209,16 @@
       <c r="P12" s="30" t="s">
         <v>46</v>
       </c>
-      <c r="Q12" s="83" t="s">
+      <c r="Q12" s="92" t="s">
         <v>48</v>
       </c>
-      <c r="R12" s="84"/>
+      <c r="R12" s="93"/>
     </row>
     <row r="13" spans="2:18" x14ac:dyDescent="0.25">
-      <c r="B13" s="72">
+      <c r="B13" s="57">
         <v>2</v>
       </c>
-      <c r="C13" s="72" t="s">
+      <c r="C13" s="57" t="s">
         <v>89</v>
       </c>
       <c r="D13" s="2" t="s">
@@ -3234,14 +3252,14 @@
       <c r="P13" s="14" t="s">
         <v>46</v>
       </c>
-      <c r="Q13" s="67" t="s">
+      <c r="Q13" s="70" t="s">
         <v>62</v>
       </c>
-      <c r="R13" s="68"/>
+      <c r="R13" s="71"/>
     </row>
     <row r="14" spans="2:18" x14ac:dyDescent="0.25">
-      <c r="B14" s="90"/>
-      <c r="C14" s="90"/>
+      <c r="B14" s="83"/>
+      <c r="C14" s="83"/>
       <c r="D14" s="2" t="s">
         <v>92</v>
       </c>
@@ -3263,12 +3281,12 @@
       <c r="N14" s="30"/>
       <c r="O14" s="30"/>
       <c r="P14" s="30"/>
-      <c r="Q14" s="83"/>
-      <c r="R14" s="84"/>
+      <c r="Q14" s="92"/>
+      <c r="R14" s="93"/>
     </row>
     <row r="15" spans="2:18" x14ac:dyDescent="0.25">
-      <c r="B15" s="90"/>
-      <c r="C15" s="90"/>
+      <c r="B15" s="83"/>
+      <c r="C15" s="83"/>
       <c r="D15" s="2" t="s">
         <v>93</v>
       </c>
@@ -3290,12 +3308,12 @@
       <c r="N15" s="30"/>
       <c r="O15" s="30"/>
       <c r="P15" s="30"/>
-      <c r="Q15" s="83"/>
-      <c r="R15" s="84"/>
+      <c r="Q15" s="92"/>
+      <c r="R15" s="93"/>
     </row>
     <row r="16" spans="2:18" x14ac:dyDescent="0.25">
-      <c r="B16" s="90"/>
-      <c r="C16" s="90"/>
+      <c r="B16" s="83"/>
+      <c r="C16" s="83"/>
       <c r="D16" s="2" t="s">
         <v>94</v>
       </c>
@@ -3311,12 +3329,12 @@
       <c r="N16" s="30"/>
       <c r="O16" s="30"/>
       <c r="P16" s="30"/>
-      <c r="Q16" s="83"/>
-      <c r="R16" s="84"/>
+      <c r="Q16" s="92"/>
+      <c r="R16" s="93"/>
     </row>
     <row r="17" spans="2:18" x14ac:dyDescent="0.25">
-      <c r="B17" s="90"/>
-      <c r="C17" s="90"/>
+      <c r="B17" s="83"/>
+      <c r="C17" s="83"/>
       <c r="D17" s="2" t="s">
         <v>95</v>
       </c>
@@ -3332,12 +3350,12 @@
       <c r="N17" s="30"/>
       <c r="O17" s="30"/>
       <c r="P17" s="30"/>
-      <c r="Q17" s="83"/>
-      <c r="R17" s="84"/>
+      <c r="Q17" s="92"/>
+      <c r="R17" s="93"/>
     </row>
     <row r="18" spans="2:18" x14ac:dyDescent="0.25">
-      <c r="B18" s="73"/>
-      <c r="C18" s="73"/>
+      <c r="B18" s="58"/>
+      <c r="C18" s="58"/>
       <c r="D18" s="2" t="s">
         <v>96</v>
       </c>
@@ -3353,14 +3371,14 @@
       <c r="N18" s="30"/>
       <c r="O18" s="30"/>
       <c r="P18" s="30"/>
-      <c r="Q18" s="83"/>
-      <c r="R18" s="84"/>
+      <c r="Q18" s="92"/>
+      <c r="R18" s="93"/>
     </row>
     <row r="19" spans="2:18" x14ac:dyDescent="0.25">
-      <c r="B19" s="72">
+      <c r="B19" s="57">
         <v>3</v>
       </c>
-      <c r="C19" s="91" t="s">
+      <c r="C19" s="84" t="s">
         <v>97</v>
       </c>
       <c r="D19" s="2" t="s">
@@ -3378,12 +3396,12 @@
       <c r="N19" s="30"/>
       <c r="O19" s="30"/>
       <c r="P19" s="30"/>
-      <c r="Q19" s="83"/>
-      <c r="R19" s="84"/>
+      <c r="Q19" s="92"/>
+      <c r="R19" s="93"/>
     </row>
     <row r="20" spans="2:18" x14ac:dyDescent="0.25">
-      <c r="B20" s="90"/>
-      <c r="C20" s="92"/>
+      <c r="B20" s="83"/>
+      <c r="C20" s="85"/>
       <c r="D20" s="2" t="s">
         <v>99</v>
       </c>
@@ -3399,12 +3417,12 @@
       <c r="N20" s="30"/>
       <c r="O20" s="30"/>
       <c r="P20" s="30"/>
-      <c r="Q20" s="83"/>
-      <c r="R20" s="84"/>
+      <c r="Q20" s="92"/>
+      <c r="R20" s="93"/>
     </row>
     <row r="21" spans="2:18" x14ac:dyDescent="0.25">
-      <c r="B21" s="90"/>
-      <c r="C21" s="92"/>
+      <c r="B21" s="83"/>
+      <c r="C21" s="85"/>
       <c r="D21" s="2" t="s">
         <v>100</v>
       </c>
@@ -3420,12 +3438,12 @@
       <c r="N21" s="30"/>
       <c r="O21" s="30"/>
       <c r="P21" s="30"/>
-      <c r="Q21" s="83"/>
-      <c r="R21" s="84"/>
+      <c r="Q21" s="92"/>
+      <c r="R21" s="93"/>
     </row>
     <row r="22" spans="2:18" x14ac:dyDescent="0.25">
-      <c r="B22" s="90"/>
-      <c r="C22" s="92"/>
+      <c r="B22" s="83"/>
+      <c r="C22" s="85"/>
       <c r="D22" s="2" t="s">
         <v>101</v>
       </c>
@@ -3441,12 +3459,12 @@
       <c r="N22" s="30"/>
       <c r="O22" s="30"/>
       <c r="P22" s="30"/>
-      <c r="Q22" s="83"/>
-      <c r="R22" s="84"/>
+      <c r="Q22" s="92"/>
+      <c r="R22" s="93"/>
     </row>
     <row r="23" spans="2:18" x14ac:dyDescent="0.25">
-      <c r="B23" s="90"/>
-      <c r="C23" s="92"/>
+      <c r="B23" s="83"/>
+      <c r="C23" s="85"/>
       <c r="D23" s="2" t="s">
         <v>102</v>
       </c>
@@ -3462,12 +3480,12 @@
       <c r="N23" s="30"/>
       <c r="O23" s="30"/>
       <c r="P23" s="30"/>
-      <c r="Q23" s="83"/>
-      <c r="R23" s="84"/>
+      <c r="Q23" s="92"/>
+      <c r="R23" s="93"/>
     </row>
     <row r="24" spans="2:18" x14ac:dyDescent="0.25">
-      <c r="B24" s="73"/>
-      <c r="C24" s="93"/>
+      <c r="B24" s="58"/>
+      <c r="C24" s="86"/>
       <c r="D24" s="2" t="s">
         <v>103</v>
       </c>
@@ -3483,14 +3501,14 @@
       <c r="N24" s="30"/>
       <c r="O24" s="30"/>
       <c r="P24" s="30"/>
-      <c r="Q24" s="83"/>
-      <c r="R24" s="84"/>
+      <c r="Q24" s="92"/>
+      <c r="R24" s="93"/>
     </row>
     <row r="25" spans="2:18" x14ac:dyDescent="0.25">
-      <c r="B25" s="72">
+      <c r="B25" s="57">
         <v>4</v>
       </c>
-      <c r="C25" s="91" t="s">
+      <c r="C25" s="84" t="s">
         <v>50</v>
       </c>
       <c r="D25" s="2" t="s">
@@ -3508,31 +3526,31 @@
       <c r="N25" s="30"/>
       <c r="O25" s="30"/>
       <c r="P25" s="30"/>
-      <c r="Q25" s="83"/>
-      <c r="R25" s="84"/>
+      <c r="Q25" s="92"/>
+      <c r="R25" s="93"/>
     </row>
     <row r="26" spans="2:18" x14ac:dyDescent="0.25">
-      <c r="B26" s="90"/>
-      <c r="C26" s="92"/>
+      <c r="B26" s="83"/>
+      <c r="C26" s="85"/>
       <c r="D26" s="2" t="s">
         <v>50</v>
       </c>
     </row>
     <row r="27" spans="2:18" x14ac:dyDescent="0.25">
-      <c r="B27" s="90"/>
-      <c r="C27" s="92"/>
+      <c r="B27" s="83"/>
+      <c r="C27" s="85"/>
       <c r="D27" s="2" t="s">
         <v>50</v>
       </c>
     </row>
     <row r="28" spans="2:18" x14ac:dyDescent="0.25">
-      <c r="B28" s="90"/>
-      <c r="C28" s="92"/>
+      <c r="B28" s="83"/>
+      <c r="C28" s="85"/>
       <c r="D28" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="G28" s="56"/>
-      <c r="H28" s="56"/>
+      <c r="G28" s="82"/>
+      <c r="H28" s="82"/>
       <c r="I28" s="88"/>
       <c r="J28" s="88"/>
       <c r="K28" s="88"/>
@@ -3541,27 +3559,51 @@
       <c r="N28" s="39"/>
     </row>
     <row r="29" spans="2:18" x14ac:dyDescent="0.25">
-      <c r="B29" s="90"/>
-      <c r="C29" s="92"/>
+      <c r="B29" s="83"/>
+      <c r="C29" s="85"/>
       <c r="D29" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="I29" s="94"/>
-      <c r="J29" s="94"/>
-      <c r="K29" s="94"/>
-      <c r="L29" s="94"/>
-      <c r="M29" s="94"/>
+      <c r="I29" s="87"/>
+      <c r="J29" s="87"/>
+      <c r="K29" s="87"/>
+      <c r="L29" s="87"/>
+      <c r="M29" s="87"/>
       <c r="N29" s="40"/>
     </row>
     <row r="30" spans="2:18" x14ac:dyDescent="0.25">
-      <c r="B30" s="73"/>
-      <c r="C30" s="93"/>
+      <c r="B30" s="58"/>
+      <c r="C30" s="86"/>
       <c r="D30" s="2" t="s">
         <v>50</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="40">
+    <mergeCell ref="Q19:R19"/>
+    <mergeCell ref="Q20:R20"/>
+    <mergeCell ref="Q21:R21"/>
+    <mergeCell ref="Q13:R13"/>
+    <mergeCell ref="K6:P6"/>
+    <mergeCell ref="Q10:R10"/>
+    <mergeCell ref="Q11:R11"/>
+    <mergeCell ref="Q12:R12"/>
+    <mergeCell ref="G28:H28"/>
+    <mergeCell ref="I28:M28"/>
+    <mergeCell ref="B5:D5"/>
+    <mergeCell ref="Q6:R6"/>
+    <mergeCell ref="H6:H7"/>
+    <mergeCell ref="Q25:R25"/>
+    <mergeCell ref="Q14:R14"/>
+    <mergeCell ref="Q15:R15"/>
+    <mergeCell ref="Q22:R22"/>
+    <mergeCell ref="Q23:R23"/>
+    <mergeCell ref="Q24:R24"/>
+    <mergeCell ref="Q16:R16"/>
+    <mergeCell ref="Q17:R17"/>
+    <mergeCell ref="Q18:R18"/>
+    <mergeCell ref="Q8:R8"/>
+    <mergeCell ref="Q9:R9"/>
     <mergeCell ref="B1:E1"/>
     <mergeCell ref="G6:G7"/>
     <mergeCell ref="I6:I7"/>
@@ -3578,30 +3620,6 @@
     <mergeCell ref="G5:R5"/>
     <mergeCell ref="B3:G3"/>
     <mergeCell ref="Q7:R7"/>
-    <mergeCell ref="G28:H28"/>
-    <mergeCell ref="I28:M28"/>
-    <mergeCell ref="B5:D5"/>
-    <mergeCell ref="Q6:R6"/>
-    <mergeCell ref="H6:H7"/>
-    <mergeCell ref="Q25:R25"/>
-    <mergeCell ref="Q14:R14"/>
-    <mergeCell ref="Q15:R15"/>
-    <mergeCell ref="Q22:R22"/>
-    <mergeCell ref="Q23:R23"/>
-    <mergeCell ref="Q24:R24"/>
-    <mergeCell ref="Q16:R16"/>
-    <mergeCell ref="Q17:R17"/>
-    <mergeCell ref="Q18:R18"/>
-    <mergeCell ref="Q8:R8"/>
-    <mergeCell ref="Q9:R9"/>
-    <mergeCell ref="Q19:R19"/>
-    <mergeCell ref="Q20:R20"/>
-    <mergeCell ref="Q21:R21"/>
-    <mergeCell ref="Q13:R13"/>
-    <mergeCell ref="K6:P6"/>
-    <mergeCell ref="Q10:R10"/>
-    <mergeCell ref="Q11:R11"/>
-    <mergeCell ref="Q12:R12"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -3614,7 +3632,7 @@
   <sheetPr>
     <tabColor theme="7" tint="-0.249977111117893"/>
   </sheetPr>
-  <dimension ref="B1:P24"/>
+  <dimension ref="B1:P31"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="6" max="6" width="14.5703125" customWidth="1"/>
@@ -3636,54 +3654,54 @@
       <c r="E1" s="54"/>
     </row>
     <row r="3" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B3" s="127" t="s">
+      <c r="B3" s="104" t="s">
         <v>104</v>
       </c>
-      <c r="C3" s="127"/>
-      <c r="D3" s="127"/>
-      <c r="E3" s="127"/>
-      <c r="F3" s="127"/>
-      <c r="G3" s="127"/>
-      <c r="H3" s="127"/>
-      <c r="I3" s="127"/>
-      <c r="J3" s="127"/>
-      <c r="K3" s="127"/>
-      <c r="L3" s="127"/>
-      <c r="M3" s="127"/>
-      <c r="N3" s="127"/>
+      <c r="C3" s="104"/>
+      <c r="D3" s="104"/>
+      <c r="E3" s="104"/>
+      <c r="F3" s="104"/>
+      <c r="G3" s="104"/>
+      <c r="H3" s="104"/>
+      <c r="I3" s="104"/>
+      <c r="J3" s="104"/>
+      <c r="K3" s="104"/>
+      <c r="L3" s="104"/>
+      <c r="M3" s="104"/>
+      <c r="N3" s="104"/>
     </row>
     <row r="4" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B4" s="79" t="s">
+      <c r="B4" s="64" t="s">
         <v>105</v>
       </c>
-      <c r="C4" s="125" t="s">
+      <c r="C4" s="102" t="s">
         <v>106</v>
       </c>
-      <c r="D4" s="111" t="s">
+      <c r="D4" s="118" t="s">
         <v>107</v>
       </c>
-      <c r="E4" s="63" t="s">
+      <c r="E4" s="78" t="s">
         <v>108</v>
       </c>
-      <c r="F4" s="61" t="s">
+      <c r="F4" s="76" t="s">
         <v>30</v>
       </c>
-      <c r="G4" s="66"/>
-      <c r="H4" s="66"/>
-      <c r="I4" s="66"/>
-      <c r="J4" s="66"/>
-      <c r="K4" s="66"/>
-      <c r="L4" s="62"/>
-      <c r="M4" s="65" t="s">
+      <c r="G4" s="81"/>
+      <c r="H4" s="81"/>
+      <c r="I4" s="81"/>
+      <c r="J4" s="81"/>
+      <c r="K4" s="81"/>
+      <c r="L4" s="77"/>
+      <c r="M4" s="80" t="s">
         <v>31</v>
       </c>
-      <c r="N4" s="65"/>
+      <c r="N4" s="80"/>
     </row>
     <row r="5" spans="2:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B5" s="110"/>
-      <c r="C5" s="126"/>
-      <c r="D5" s="112"/>
-      <c r="E5" s="124"/>
+      <c r="B5" s="117"/>
+      <c r="C5" s="103"/>
+      <c r="D5" s="119"/>
+      <c r="E5" s="101"/>
       <c r="F5" s="22" t="s">
         <v>128</v>
       </c>
@@ -3699,10 +3717,10 @@
       <c r="J5" s="22" t="s">
         <v>132</v>
       </c>
-      <c r="K5" s="122" t="s">
+      <c r="K5" s="97" t="s">
         <v>133</v>
       </c>
-      <c r="L5" s="123"/>
+      <c r="L5" s="98"/>
       <c r="M5" s="22" t="s">
         <v>39</v>
       </c>
@@ -3714,7 +3732,7 @@
       <c r="B6" s="20">
         <v>1</v>
       </c>
-      <c r="C6" s="108" t="s">
+      <c r="C6" s="115" t="s">
         <v>110</v>
       </c>
       <c r="D6" s="26" t="s">
@@ -3738,10 +3756,10 @@
       <c r="J6" s="25">
         <v>40</v>
       </c>
-      <c r="K6" s="97" t="s">
+      <c r="K6" s="95" t="s">
         <v>138</v>
       </c>
-      <c r="L6" s="98" t="s">
+      <c r="L6" s="96" t="s">
         <v>47</v>
       </c>
       <c r="M6" s="25" t="s">
@@ -3756,7 +3774,7 @@
         <f>B6+1</f>
         <v>2</v>
       </c>
-      <c r="C7" s="108"/>
+      <c r="C7" s="115"/>
       <c r="D7" s="27" t="s">
         <v>134</v>
       </c>
@@ -3778,10 +3796,10 @@
       <c r="J7" s="50">
         <v>15</v>
       </c>
-      <c r="K7" s="95" t="s">
+      <c r="K7" s="99" t="s">
         <v>138</v>
       </c>
-      <c r="L7" s="96" t="s">
+      <c r="L7" s="100" t="s">
         <v>139</v>
       </c>
       <c r="M7" s="50" t="s">
@@ -3795,7 +3813,7 @@
       <c r="B8" s="9">
         <v>3</v>
       </c>
-      <c r="C8" s="108"/>
+      <c r="C8" s="115"/>
       <c r="D8" s="27" t="s">
         <v>112</v>
       </c>
@@ -3817,10 +3835,10 @@
       <c r="J8" s="50">
         <v>15</v>
       </c>
-      <c r="K8" s="95" t="s">
+      <c r="K8" s="99" t="s">
         <v>138</v>
       </c>
-      <c r="L8" s="96" t="s">
+      <c r="L8" s="100" t="s">
         <v>140</v>
       </c>
       <c r="M8" s="50" t="s">
@@ -3834,7 +3852,7 @@
       <c r="B9" s="9">
         <v>4</v>
       </c>
-      <c r="C9" s="108"/>
+      <c r="C9" s="115"/>
       <c r="D9" s="27" t="s">
         <v>135</v>
       </c>
@@ -3856,10 +3874,10 @@
       <c r="J9" s="50">
         <v>15</v>
       </c>
-      <c r="K9" s="95" t="s">
+      <c r="K9" s="99" t="s">
         <v>138</v>
       </c>
-      <c r="L9" s="96" t="s">
+      <c r="L9" s="100" t="s">
         <v>141</v>
       </c>
       <c r="M9" s="50" t="s">
@@ -3873,7 +3891,7 @@
       <c r="B10" s="20">
         <v>5</v>
       </c>
-      <c r="C10" s="108"/>
+      <c r="C10" s="115"/>
       <c r="D10" s="27" t="s">
         <v>113</v>
       </c>
@@ -3895,10 +3913,10 @@
       <c r="J10" s="50">
         <v>300</v>
       </c>
-      <c r="K10" s="95" t="s">
+      <c r="K10" s="99" t="s">
         <v>152</v>
       </c>
-      <c r="L10" s="96" t="s">
+      <c r="L10" s="100" t="s">
         <v>140</v>
       </c>
       <c r="M10" s="50" t="s">
@@ -3912,7 +3930,7 @@
       <c r="B11" s="9">
         <v>6</v>
       </c>
-      <c r="C11" s="108"/>
+      <c r="C11" s="115"/>
       <c r="D11" s="27" t="s">
         <v>136</v>
       </c>
@@ -3934,10 +3952,10 @@
       <c r="J11" s="50">
         <v>300</v>
       </c>
-      <c r="K11" s="95" t="s">
+      <c r="K11" s="99" t="s">
         <v>153</v>
       </c>
-      <c r="L11" s="96" t="s">
+      <c r="L11" s="100" t="s">
         <v>141</v>
       </c>
       <c r="M11" s="50" t="s">
@@ -3951,7 +3969,7 @@
       <c r="B12" s="9">
         <v>7</v>
       </c>
-      <c r="C12" s="108"/>
+      <c r="C12" s="115"/>
       <c r="D12" s="27" t="s">
         <v>154</v>
       </c>
@@ -3973,10 +3991,10 @@
       <c r="J12" s="50">
         <v>15</v>
       </c>
-      <c r="K12" s="95" t="s">
+      <c r="K12" s="99" t="s">
         <v>138</v>
       </c>
-      <c r="L12" s="96" t="s">
+      <c r="L12" s="100" t="s">
         <v>142</v>
       </c>
       <c r="M12" s="50" t="s">
@@ -3990,7 +4008,7 @@
       <c r="B13" s="9">
         <v>8</v>
       </c>
-      <c r="C13" s="108"/>
+      <c r="C13" s="115"/>
       <c r="D13" s="27" t="s">
         <v>52</v>
       </c>
@@ -4012,10 +4030,10 @@
       <c r="J13" s="50">
         <v>15</v>
       </c>
-      <c r="K13" s="95" t="s">
+      <c r="K13" s="99" t="s">
         <v>138</v>
       </c>
-      <c r="L13" s="96" t="s">
+      <c r="L13" s="100" t="s">
         <v>143</v>
       </c>
       <c r="M13" s="50" t="s">
@@ -4029,7 +4047,7 @@
       <c r="B14" s="20">
         <v>9</v>
       </c>
-      <c r="C14" s="108"/>
+      <c r="C14" s="115"/>
       <c r="D14" s="27" t="s">
         <v>52</v>
       </c>
@@ -4051,10 +4069,10 @@
       <c r="J14" s="50">
         <v>15</v>
       </c>
-      <c r="K14" s="95" t="s">
+      <c r="K14" s="99" t="s">
         <v>138</v>
       </c>
-      <c r="L14" s="96" t="s">
+      <c r="L14" s="100" t="s">
         <v>144</v>
       </c>
       <c r="M14" s="50" t="s">
@@ -4068,7 +4086,7 @@
       <c r="B15" s="20">
         <v>10</v>
       </c>
-      <c r="C15" s="108"/>
+      <c r="C15" s="115"/>
       <c r="D15" s="48"/>
       <c r="E15" s="9" t="s">
         <v>114</v>
@@ -4088,10 +4106,10 @@
       <c r="J15" s="50">
         <v>15</v>
       </c>
-      <c r="K15" s="97" t="s">
+      <c r="K15" s="95" t="s">
         <v>138</v>
       </c>
-      <c r="L15" s="98" t="s">
+      <c r="L15" s="96" t="s">
         <v>145</v>
       </c>
       <c r="M15" s="49" t="s">
@@ -4105,7 +4123,7 @@
       <c r="B16" s="9">
         <v>11</v>
       </c>
-      <c r="C16" s="109"/>
+      <c r="C16" s="116"/>
       <c r="D16" s="28" t="s">
         <v>50</v>
       </c>
@@ -4127,10 +4145,10 @@
       <c r="J16" s="50">
         <v>15</v>
       </c>
-      <c r="K16" s="97" t="s">
+      <c r="K16" s="95" t="s">
         <v>138</v>
       </c>
-      <c r="L16" s="98" t="s">
+      <c r="L16" s="96" t="s">
         <v>146</v>
       </c>
       <c r="M16" s="21" t="s">
@@ -4167,98 +4185,98 @@
       <c r="H18" s="5"/>
       <c r="I18" s="5"/>
       <c r="J18" s="5"/>
-      <c r="K18" s="107"/>
-      <c r="L18" s="107"/>
+      <c r="K18" s="127"/>
+      <c r="L18" s="127"/>
       <c r="M18" s="5"/>
     </row>
     <row r="19" spans="2:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="M19" s="5"/>
     </row>
     <row r="20" spans="2:16" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="C20" s="101" t="s">
+      <c r="C20" s="106" t="s">
         <v>117</v>
       </c>
-      <c r="D20" s="103"/>
-      <c r="E20" s="103"/>
-      <c r="F20" s="104"/>
+      <c r="D20" s="107"/>
+      <c r="E20" s="107"/>
+      <c r="F20" s="108"/>
       <c r="G20" s="35" t="s">
         <v>118</v>
       </c>
-      <c r="H20" s="101" t="s">
+      <c r="H20" s="106" t="s">
         <v>119</v>
       </c>
-      <c r="I20" s="102"/>
-      <c r="J20" s="103"/>
-      <c r="K20" s="103"/>
-      <c r="L20" s="104"/>
-      <c r="M20" s="101" t="s">
+      <c r="I20" s="109"/>
+      <c r="J20" s="107"/>
+      <c r="K20" s="107"/>
+      <c r="L20" s="108"/>
+      <c r="M20" s="106" t="s">
         <v>120</v>
       </c>
-      <c r="N20" s="102"/>
-      <c r="O20" s="103"/>
-      <c r="P20" s="104"/>
+      <c r="N20" s="109"/>
+      <c r="O20" s="107"/>
+      <c r="P20" s="108"/>
     </row>
     <row r="21" spans="2:16" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B21" s="115" t="s">
+      <c r="B21" s="122" t="s">
         <v>106</v>
       </c>
-      <c r="C21" s="116" t="s">
+      <c r="C21" s="123" t="s">
         <v>121</v>
       </c>
-      <c r="D21" s="100" t="s">
+      <c r="D21" s="105" t="s">
         <v>122</v>
       </c>
-      <c r="E21" s="100" t="s">
+      <c r="E21" s="105" t="s">
         <v>123</v>
       </c>
-      <c r="F21" s="99" t="s">
+      <c r="F21" s="124" t="s">
         <v>124</v>
       </c>
-      <c r="G21" s="121" t="s">
+      <c r="G21" s="114" t="s">
         <v>125</v>
       </c>
-      <c r="H21" s="117" t="s">
+      <c r="H21" s="110" t="s">
         <v>126</v>
       </c>
-      <c r="I21" s="118"/>
-      <c r="J21" s="100" t="s">
+      <c r="I21" s="111"/>
+      <c r="J21" s="105" t="s">
         <v>121</v>
       </c>
-      <c r="K21" s="100" t="s">
+      <c r="K21" s="105" t="s">
         <v>122</v>
       </c>
-      <c r="L21" s="99" t="s">
+      <c r="L21" s="124" t="s">
         <v>123</v>
       </c>
-      <c r="M21" s="105" t="s">
+      <c r="M21" s="125" t="s">
         <v>126</v>
       </c>
-      <c r="N21" s="100" t="s">
+      <c r="N21" s="105" t="s">
         <v>121</v>
       </c>
-      <c r="O21" s="100" t="s">
+      <c r="O21" s="105" t="s">
         <v>122</v>
       </c>
-      <c r="P21" s="99" t="s">
+      <c r="P21" s="124" t="s">
         <v>123</v>
       </c>
     </row>
     <row r="22" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B22" s="115"/>
-      <c r="C22" s="116"/>
-      <c r="D22" s="100"/>
-      <c r="E22" s="100"/>
-      <c r="F22" s="99"/>
-      <c r="G22" s="121"/>
-      <c r="H22" s="119"/>
-      <c r="I22" s="120"/>
-      <c r="J22" s="100"/>
-      <c r="K22" s="100"/>
-      <c r="L22" s="99"/>
-      <c r="M22" s="106"/>
-      <c r="N22" s="100"/>
-      <c r="O22" s="100"/>
-      <c r="P22" s="99"/>
+      <c r="B22" s="122"/>
+      <c r="C22" s="123"/>
+      <c r="D22" s="105"/>
+      <c r="E22" s="105"/>
+      <c r="F22" s="124"/>
+      <c r="G22" s="114"/>
+      <c r="H22" s="112"/>
+      <c r="I22" s="113"/>
+      <c r="J22" s="105"/>
+      <c r="K22" s="105"/>
+      <c r="L22" s="124"/>
+      <c r="M22" s="126"/>
+      <c r="N22" s="105"/>
+      <c r="O22" s="105"/>
+      <c r="P22" s="124"/>
     </row>
     <row r="23" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B23" s="38" t="s">
@@ -4275,10 +4293,10 @@
       </c>
       <c r="F23" s="37"/>
       <c r="G23" s="42"/>
-      <c r="H23" s="113" t="s">
+      <c r="H23" s="120" t="s">
         <v>127</v>
       </c>
-      <c r="I23" s="114"/>
+      <c r="I23" s="121"/>
       <c r="J23" s="2">
         <v>0</v>
       </c>
@@ -4304,8 +4322,60 @@
     <row r="24" spans="2:16" x14ac:dyDescent="0.25">
       <c r="M24" s="3"/>
     </row>
+    <row r="26" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="B26" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="27" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="B27" t="s">
+        <v>158</v>
+      </c>
+      <c r="D27" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="28" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="D28" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="29" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="D29" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="31" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="B31" t="s">
+        <v>157</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="40">
+    <mergeCell ref="K10:L10"/>
+    <mergeCell ref="K15:L15"/>
+    <mergeCell ref="L21:L22"/>
+    <mergeCell ref="O21:O22"/>
+    <mergeCell ref="P21:P22"/>
+    <mergeCell ref="M20:P20"/>
+    <mergeCell ref="M21:M22"/>
+    <mergeCell ref="N21:N22"/>
+    <mergeCell ref="K18:L18"/>
+    <mergeCell ref="C6:C16"/>
+    <mergeCell ref="B4:B5"/>
+    <mergeCell ref="D4:D5"/>
+    <mergeCell ref="H23:I23"/>
+    <mergeCell ref="B21:B22"/>
+    <mergeCell ref="C21:C22"/>
+    <mergeCell ref="D21:D22"/>
+    <mergeCell ref="E21:E22"/>
+    <mergeCell ref="F21:F22"/>
+    <mergeCell ref="J21:J22"/>
+    <mergeCell ref="C20:F20"/>
+    <mergeCell ref="H20:L20"/>
+    <mergeCell ref="H21:I22"/>
+    <mergeCell ref="G21:G22"/>
+    <mergeCell ref="K21:K22"/>
     <mergeCell ref="B1:E1"/>
     <mergeCell ref="K16:L16"/>
     <mergeCell ref="M4:N4"/>
@@ -4322,30 +4392,6 @@
     <mergeCell ref="B3:N3"/>
     <mergeCell ref="K8:L8"/>
     <mergeCell ref="K9:L9"/>
-    <mergeCell ref="J21:J22"/>
-    <mergeCell ref="C20:F20"/>
-    <mergeCell ref="H20:L20"/>
-    <mergeCell ref="H21:I22"/>
-    <mergeCell ref="G21:G22"/>
-    <mergeCell ref="K21:K22"/>
-    <mergeCell ref="C6:C16"/>
-    <mergeCell ref="B4:B5"/>
-    <mergeCell ref="D4:D5"/>
-    <mergeCell ref="H23:I23"/>
-    <mergeCell ref="B21:B22"/>
-    <mergeCell ref="C21:C22"/>
-    <mergeCell ref="D21:D22"/>
-    <mergeCell ref="E21:E22"/>
-    <mergeCell ref="F21:F22"/>
-    <mergeCell ref="K10:L10"/>
-    <mergeCell ref="K15:L15"/>
-    <mergeCell ref="L21:L22"/>
-    <mergeCell ref="O21:O22"/>
-    <mergeCell ref="P21:P22"/>
-    <mergeCell ref="M20:P20"/>
-    <mergeCell ref="M21:M22"/>
-    <mergeCell ref="N21:N22"/>
-    <mergeCell ref="K18:L18"/>
   </mergeCells>
   <phoneticPr fontId="28" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -4355,18 +4401,18 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
   <Edit>DocumentLibraryForm</Edit>
   <New>DocumentLibraryForm</New>
 </FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -4514,18 +4560,18 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FF0EB622-FDCF-4321-9FF5-C0B282D1670E}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2BC1EB47-4FFF-47F3-894F-DED91590EA19}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2BC1EB47-4FFF-47F3-894F-DED91590EA19}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FF0EB622-FDCF-4321-9FF5-C0B282D1670E}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>